<commit_message>
feat(F-NAR-019): polish TREE-DIF-003 et TREE-DIF-020 xlsx
Alignement xlsx sur merged vocal après re-apply.
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-003.xlsx
+++ b/stories/arbres/TREE-DIF-003.xlsx
@@ -1197,17 +1197,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un éclat de thym colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois.</t>
+          <t>La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. La casserole frémit, près du thym. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un éclat de thym colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un &lt;emphasis level="moderate"&gt;éclat de thym&lt;/emphasis&gt; colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. La casserole frémit, près du thym. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un &lt;emphasis level="moderate"&gt;éclat de thym&lt;/emphasis&gt; colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un &lt;emphasis&gt;éclat de thym&lt;/emphasis&gt; colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois. [pause]</t>
+          <t>La gouttière compte, goutte après goutte. Mila compte avec elle, dans la cuisine. Ça sent le poireau, et le thym coupé. La casserole frémit, près du thym. Un nuage de soupe cache la vitre. Je fais un rond, pour voir. Papa essuie, et le seuil apparaît. Le manteau à pois goutte, au crochet. Un &lt;emphasis&gt;éclat de thym&lt;/emphasis&gt; colle à un pois. Il n'était pas là, ce matin. C'est le thym de la soupe. En ce moment, Mila touche le pois. Je sors, avant la dernière goutte. Elle veut le manteau, et les lunettes. Le seau attend sous l'évier. Aniss pousse la porte, sans un mot. Il s'arrête, et regarde l'éclat. On y va, Aniss. Aniss ne dit rien. Merci, tu as attendu sa voix. Le thym, moi je le vois. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1344,6 +1344,7 @@
           <t>narrateur|La gouttière compte, goutte après goutte.
 narrateur|Mila compte avec elle, dans la cuisine.
 narrateur|Ça sent le poireau, et le thym coupé.
+narrateur|La casserole frémit, près du thym.
 narrateur|Un nuage de soupe cache la vitre.
 papa|Je fais un rond, pour voir.
 narrateur|Papa essuie, et le seuil apparaît.
@@ -1968,17 +1969,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, sur un pois.</t>
+          <t>Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, sur un pois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, sur un pois.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, sur un pois.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, sur un pois. [pause]</t>
+          <t>Le manteau reste sur elle, un peu lourd. La feuille est dans la poche. Les lunettes tiennent, Mila ? Oui, sur mon nez. Le seau, Aniss le tient. J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, sur un pois. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2120,6 +2121,8 @@
 enfant-m|J'ai l'anse.
 narrateur|Ils avancent vers le seuil, sans courir.
 maman|La gouttière n'a pas fini.
+enfant-f|Une maison, avant la dernière goutte.
+narrateur|Aniss marche derrière, sans se presser.
 narrateur|Un éclat de thym brille, sur un pois.</t>
         </is>
       </c>
@@ -7249,17 +7252,17 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Les lunettes restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord d'un verre.</t>
+          <t>Les lunettes restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord d'un verre.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt; restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord d'un verre.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Les &lt;emphasis level="moderate"&gt;lunettes&lt;/emphasis&gt; restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord d'un verre.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Les &lt;emphasis&gt;lunettes&lt;/emphasis&gt; restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord d'un verre. [pause]</t>
+          <t>Les &lt;emphasis&gt;lunettes&lt;/emphasis&gt; restent nettes, sur son nez. Je vois le seuil, dehors. Le manteau te tient chaud ? Oui, il est un peu lourd. Aniss, tu tiens le seau ? J'ai l'anse. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord d'un verre. [pause]</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
@@ -7401,6 +7404,8 @@
 enfant-m|J'ai l'anse.
 narrateur|Ils avancent vers le seuil, sans courir.
 papa|La gouttière n'a pas fini.
+enfant-f|Une maison, avant la dernière goutte.
+narrateur|Aniss marche derrière, sans se presser.
 narrateur|Un éclat de thym brille, au bord d'un verre.</t>
         </is>
       </c>
@@ -12150,17 +12155,17 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Mila attrape le seau sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ?</t>
+          <t>Mila attrape le seau sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ? Oui.</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila attrape le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ?&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila attrape le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Mila attrape le &lt;emphasis&gt;seau&lt;/emphasis&gt; sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ? [pause]</t>
+          <t>Mila attrape le &lt;emphasis&gt;seau&lt;/emphasis&gt; sous l'évier. Il sonne creux, comme un petit tambour. Il est coincé ! Je tire, moi. Aniss pose les deux mains, et attend. Mila veut tirer trop fort, trop vite. Deux mains, et on glisse. Le seau se libère, d'un coup. C'est l'hôtel. Une feuille, et une goutte ? Mila pose une feuille sèche, au fond. Le manteau, et les lunettes aussi ? Oui, on les prend. Je porte l'anse. Le seau se balance, puis se tient. L'hôtel est prêt ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
@@ -12309,7 +12314,8 @@
 enfant-f|Oui, on les prend.
 enfant-m|Je porte l'anse.
 narrateur|Le seau se balance, puis se tient.
-maman|L'hôtel est prêt ?</t>
+maman|L'hôtel est prêt ?
+enfant-f|Oui.</t>
         </is>
       </c>
       <c r="AX60" t="inlineStr">
@@ -12529,17 +12535,17 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord du seau.</t>
+          <t>La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord du seau.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord du &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord du &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Un éclat de thym brille, au bord du &lt;emphasis&gt;seau&lt;/emphasis&gt;. [pause]</t>
+          <t>La feuille nage dans sa goutte, au fond. L'hôtel voyage. Deux mains sur l'anse, Aniss. J'ai. Le manteau te tient, Mila ? Oui, et les lunettes. Ils avancent vers le seuil, sans courir. La gouttière n'a pas fini. Une maison, avant la dernière goutte. Aniss marche derrière, sans se presser. Un éclat de thym brille, au bord du &lt;emphasis&gt;seau&lt;/emphasis&gt;. [pause]</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
@@ -12681,6 +12687,8 @@
 enfant-f|Oui, et les lunettes.
 narrateur|Ils avancent vers le seuil, sans courir.
 papa|La gouttière n'a pas fini.
+enfant-f|Une maison, avant la dernière goutte.
+narrateur|Aniss marche derrière, sans se presser.
 narrateur|Un éclat de thym brille, au bord du seau.</t>
         </is>
       </c>
@@ -17424,7 +17432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17502,6 +17510,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>